<commit_message>
Add revenue/sales growth guidance to Abbott guidance workbook
Enrich the By Fiscal Year tab (and Guidance Timeline) with full-year
sales-growth guidance and the basis it was measured on:

- New 'Sales Growth Guidance' and 'Sales Growth Basis' columns, color-coded
- Populate the COVID years (2021-2023) with Abbott's base-business
  ex-COVID descriptors (high single digits -> low double digits), which
  were the only top-line guidance given in those years
- Clean numeric organic ranges for FY2020 and FY2024-2026; 'comparable'
  basis flagged for FY2026 Q1 (Exact Sciences/FX)
- Updated Q3'22 COVID-testing-sales assumption to ~$7.8B
- Expanded Notes with a guide to reading the sales-growth basis

https://claude.ai/code/session_01EKrf5kyJ9fDoQd1dRoC1pG
</commit_message>
<xml_diff>
--- a/Abbott_Guidance_By_Quarter_2020-2026.xlsx
+++ b/Abbott_Guidance_By_Quarter_2020-2026.xlsx
@@ -63,7 +63,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -77,12 +77,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EEF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF3FB"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,11 +98,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,6 +113,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -185,23 +190,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -229,19 +234,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -254,13 +248,27 @@
     <xf numFmtId="164" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -279,13 +287,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -651,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -663,10 +672,11 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -679,7 +689,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How Abbott's full-year outlook was set and revised at each quarterly earnings report, Q4 2019 report (initial FY2020) through Q1 2026.  Compiled from Abbott press releases &amp; SEC 8-K exhibits.</t>
+          <t>How Abbott's full-year outlook (EPS and sales growth) was set and revised at each quarterly earnings report, Q4 2019 report (initial FY2020) through Q1 2026.  Compiled from Abbott press releases &amp; SEC 8-K exhibits.</t>
         </is>
       </c>
     </row>
@@ -731,26 +741,31 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Organic / Comparable Sales Growth</t>
+          <t>Sales Growth Guidance</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
+          <t>Sales Growth Basis</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
           <t>COVID-19 Testing Sales Assumption</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Key Commentary</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>2020-01-22</t>
@@ -795,23 +810,28 @@
           <t>7.0% – 8.0%</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>n/a (pre-COVID)</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Initial FY2020 outlook issued pre-COVID; double-digit EPS growth at midpoint.</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/0000001800/000110465920005717/tm205456d1_ex99-1.htm</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>2020-04-16</t>
@@ -827,7 +847,7 @@
           <t>FY2020</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Withdrawn</t>
         </is>
@@ -850,23 +870,28 @@
           <t>Withdrawn</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Uncertain</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Suspended all FY2020 guidance due to COVID-19 uncertainty; no new numbers provided.</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-first-quarter-2020-results-301041836.html</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>2020-07-16</t>
@@ -882,7 +907,7 @@
           <t>FY2020</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Reinstated (floor)</t>
         </is>
@@ -904,26 +929,31 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
+          <t>Not provided (EPS floor only)</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Ramping</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Guidance reinstated as an 'at least' floor given COVID uncertainty; ~$1.25 of specified items.</t>
-        </is>
-      </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
+          <t>Guidance reinstated as an 'at least' EPS floor given COVID uncertainty; no sales-growth % given; ~$1.25 of specified items.</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-second-quarter-2020-results-exceeds-analysts-expectations-301094737.html</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>2020-10-21</t>
@@ -939,7 +969,7 @@
           <t>FY2020</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
@@ -961,26 +991,31 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
+          <t>Not provided (EPS floor only)</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Strong (BinaxNOW / ID NOW / Panbio)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Raised from 'at least $3.25' on strong COVID diagnostics demand. FY2020 actual landed at $3.65 adj.</t>
-        </is>
-      </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
+          <t>Raised EPS floor from 'at least $3.25' on strong COVID diagnostics demand; no sales-growth %. FY2020 actual landed at $3.65 adj.</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
           <t>https://abbott.mediaroom.com/2020-10-21-Abbott-Reports-Third-Quarter-2020-Results-Achieves-Strong-Double-Digit-Earnings-Growth-and-Raises-Guidance</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>2021-01-27</t>
@@ -1018,26 +1053,31 @@
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>Double-digit (qualitative)</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
+          <t>~Double-digit (qualitative; no % issued)</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
         <is>
           <t>~$2.4B in Q4'20</t>
         </is>
       </c>
-      <c r="L9" s="11" t="inlineStr">
-        <is>
-          <t>Initial FY2021 outlook: EPS growth of more than 35% vs prior year on COVID-testing boom.</t>
-        </is>
-      </c>
       <c r="M9" s="11" t="inlineStr">
         <is>
+          <t>Initial FY2021 outlook: EPS growth of more than 35%. Headline was 'strong double-digit growth' but no numeric full-year sales range was issued (~3.5% favorable FX noted).</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-fourth-quarter-2020-results-issues-strong-double-digit-growth-forecast-for-2021-301216123.html</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>2021-04-20</t>
@@ -1078,23 +1118,28 @@
           <t>Not provided (qualitative)</t>
         </is>
       </c>
-      <c r="K10" s="11" t="inlineStr">
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="L10" s="11" t="inlineStr">
-        <is>
-          <t>Guidance maintained unchanged ('growth of more than 35%').</t>
-        </is>
-      </c>
       <c r="M10" s="11" t="inlineStr">
         <is>
+          <t>Guidance maintained; no numeric full-year sales-growth range issued.</t>
+        </is>
+      </c>
+      <c r="N10" s="11" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-first-quarter-2021-results-301272437.html</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>2021-07-22</t>
@@ -1136,26 +1181,31 @@
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>Sharp decline</t>
         </is>
       </c>
-      <c r="L11" s="11" t="inlineStr">
-        <is>
-          <t>Lowered on sharp drop in COVID-19 testing demand. (Abbott pre-announced a cut to 'at least $4.30' in mid-June 2021.)</t>
-        </is>
-      </c>
       <c r="M11" s="11" t="inlineStr">
         <is>
+          <t>EPS lowered on falling COVID-test demand; full-year base-business organic framed as 'low double digits' (first numerically labeled at the Jun 1, 2021 off-cycle update).</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-second-quarter-2021-results-301339347.html</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>2021-10-20</t>
@@ -1171,7 +1221,7 @@
           <t>FY2021</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
@@ -1197,26 +1247,31 @@
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>Renewed (Delta wave)</t>
         </is>
       </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>Raised sharply (~38.4% growth at midpoint) on renewed COVID-testing demand plus base-business strength.</t>
-        </is>
-      </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
+          <t>EPS raised sharply (~38.4% growth at midpoint) on renewed COVID-testing demand plus base-business strength; base organic 'low double digits' maintained.</t>
+        </is>
+      </c>
+      <c r="N12" s="11" t="inlineStr">
+        <is>
           <t>https://abbott.mediaroom.com/2021-10-20-Abbott-Reports-Third-Quarter-2021-Results-Achieves-Strong-Double-Digit-Earnings-Growth-and-Raises-Guidance</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>2022-01-26</t>
@@ -1254,26 +1309,31 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Not stated as single number</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
+          <t>High single digits</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>~$2.5B (initial)</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Initial FY2022 outlook with an initial COVID-testing sales forecast of ~$2.5B, to be updated quarterly.</t>
-        </is>
-      </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
+          <t>Initial FY2022 outlook; base-business organic 'high single digits'. Initial COVID-testing sales forecast ~$2.5B, to be updated quarterly.</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-strong-fourth-quarter-2021-results-issues-2022-forecast-301468554.html</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>2022-04-20</t>
@@ -1311,26 +1371,31 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Not stated as single number</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
+          <t>High single digits</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Raised to ~$4.5B</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Adjusted EPS maintained; COVID-testing sales forecast raised to ~$4.5B (Q1 COVID test sales $3.3B).</t>
-        </is>
-      </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
+          <t>Adjusted EPS maintained; base-business organic 'high single digits'. COVID-testing sales forecast raised to ~$4.5B (Q1 COVID test sales $3.3B).</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-first-quarter-2022-results-301528820.html</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="58" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>2022-07-20</t>
@@ -1346,7 +1411,7 @@
           <t>FY2022</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
@@ -1368,26 +1433,31 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Low double digits (base business)</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Raised to $6.1B</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>EPS raised (&gt;= $4.70 -&gt; &gt;= $4.90); COVID-testing sales raised to $6.1B; strong base business.</t>
-        </is>
-      </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
+          <t>EPS raised (&gt;= $4.70 -&gt; &gt;= $4.90); base-business organic raised to 'low double digits'; COVID-testing sales raised to $6.1B.</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-second-quarter-2022-results-and-raises-full-year-eps-guidance-301590017.html</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="58" customHeight="1">
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>2022-10-19</t>
@@ -1403,7 +1473,7 @@
           <t>FY2022</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
@@ -1429,26 +1499,31 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Double-digit base business</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>~$6.1–6.4B (implied)</t>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>EPS raised again to a defined range. FY2022 actual landed at $5.34 adj.</t>
+          <t>Raised to ~$7.8B</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
+          <t>EPS raised again to a defined range; base-business organic 'low double digits' maintained. FY2022 actual landed at $5.34 adj.</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-third-quarter-2022-results-and-raises-full-year-eps-guidance-301653429.html</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="58" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>2023-01-25</t>
@@ -1490,26 +1565,31 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>High-single digits (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
+          <t>High single digits</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>~$2.0B</t>
         </is>
       </c>
-      <c r="L17" s="11" t="inlineStr">
-        <is>
-          <t>Initial FY2023 outlook; assumed ~$2.0B of COVID-testing sales for the year.</t>
-        </is>
-      </c>
       <c r="M17" s="11" t="inlineStr">
         <is>
+          <t>Initial FY2023 outlook; base-business organic 'high single digits' ex-COVID. Assumed ~$2.0B of COVID-testing sales.</t>
+        </is>
+      </c>
+      <c r="N17" s="11" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-fourth-quarter-and-full-year-2022-results-issues-2023-financial-outlook-301730346.html</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="58" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>2023-04-19</t>
@@ -1551,26 +1631,31 @@
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>At least high-single digits (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
+          <t>≈High single digits (raised outlook)</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
         <is>
           <t>Lowered to ~$1.5B</t>
         </is>
       </c>
-      <c r="L18" s="11" t="inlineStr">
-        <is>
-          <t>Adjusted EPS maintained; higher base-business outlook offset by lower COVID. Q1 base organic +10.0%.</t>
-        </is>
-      </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
+          <t>Adjusted EPS maintained; underlying base-business outlook raised (~high single digits), offset by lower COVID. Q1 base organic +10.0%.</t>
+        </is>
+      </c>
+      <c r="N18" s="11" t="inlineStr">
+        <is>
           <t>https://abbott.mediaroom.com/2023-04-19-Abbott-Reports-First-Quarter-2023-Results-Increases-Outlook-For-Underlying-Base-Business</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="58" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>2023-07-20</t>
@@ -1612,26 +1697,31 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>Low double digits (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
         <is>
           <t>Lowered to ~$1.3B</t>
         </is>
       </c>
-      <c r="L19" s="11" t="inlineStr">
-        <is>
-          <t>Adjusted EPS maintained; base-business outlook raised again, offset by lower COVID. Q2 base organic +11.5%.</t>
-        </is>
-      </c>
       <c r="M19" s="11" t="inlineStr">
         <is>
+          <t>Adjusted EPS maintained; base-business outlook raised to 'low double digits', offset by lower COVID. Q2 base organic +11.5%.</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-second-quarter-2023-results-increases-outlook-for-underlying-base-business-301882027.html</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="58" customHeight="1">
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
           <t>2023-10-18</t>
@@ -1673,26 +1763,31 @@
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>Low double digits (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="inlineStr">
         <is>
           <t>~$1.6B (implied)</t>
         </is>
       </c>
-      <c r="L20" s="11" t="inlineStr">
-        <is>
-          <t>EPS range narrowed and midpoint raised; base-business growth maintained.</t>
-        </is>
-      </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
+          <t>EPS range narrowed and midpoint raised; base-business organic 'low double digits' maintained.</t>
+        </is>
+      </c>
+      <c r="N20" s="11" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-third-quarter-2023-results-and-raises-midpoint-of-full-year-eps-guidance-range-301960446.html</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="58" customHeight="1">
+    <row r="21" ht="60" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>2024-01-24</t>
@@ -1734,26 +1829,31 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>8.0% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
+          <t>8.0% – 10.0%</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Minimal</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Initial FY2024 outlook.</t>
-        </is>
-      </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
+          <t>Initial FY2024 outlook; headline reverts to a single organic range now that COVID is immaterial.</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-fourth-quarter-and-full-year-2023-results-issues-2024-financial-outlook-302043275.html</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="58" customHeight="1">
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>2024-04-17</t>
@@ -1769,7 +1869,7 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Raised midpoint</t>
         </is>
@@ -1795,26 +1895,31 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>8.5% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
+          <t>8.5% – 10.0%</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Minimal</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Raised midpoint of all ranges; narrowed organic range by raising the low end.</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-first-quarter-2024-results-and-raises-midpoint-of-full-year-guidance-ranges-302119393.html</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="58" customHeight="1">
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>2024-07-18</t>
@@ -1830,7 +1935,7 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
@@ -1856,26 +1961,31 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>9.5% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
+          <t>9.5% – 10.0%</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Minimal</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Raised full-year guidance again.</t>
-        </is>
-      </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
+          <t>Raised full-year guidance again; organic range narrowed upward.</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-second-quarter-2024-results-and-raises-full-year-guidance-302200584.html</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="58" customHeight="1">
+    <row r="24" ht="60" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>2024-10-16</t>
@@ -1891,7 +2001,7 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Raised midpoint / narrowed</t>
         </is>
@@ -1917,26 +2027,31 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>9.5% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
+          <t>9.5% – 10.0%</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>Minimal</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Raised midpoint / narrowed EPS; organic range maintained.</t>
-        </is>
-      </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
+          <t>Raised EPS midpoint / narrowed; organic range maintained. FY actual landed at the upper end.</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-third-quarter-2024-results-and-raises-midpoint-of-full-year-eps-guidance-range-302277755.html</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="58" customHeight="1">
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>2025-01-22</t>
@@ -1981,23 +2096,28 @@
           <t>7.5% – 8.5%</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>
       </c>
-      <c r="L25" s="11" t="inlineStr">
+      <c r="M25" s="11" t="inlineStr">
         <is>
           <t>Initial FY2025 outlook; double-digit EPS growth at midpoint; adj. operating margin 23.5%-24.0%. GAAP EPS guidance discontinued.</t>
         </is>
       </c>
-      <c r="M25" s="11" t="inlineStr">
+      <c r="N25" s="11" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-fourth-quarter-and-full-year-2024-results-issues-2025-financial-outlook-302357321.html</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="58" customHeight="1">
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
           <t>2025-04-16</t>
@@ -2042,23 +2162,28 @@
           <t>7.5% – 8.5%</t>
         </is>
       </c>
-      <c r="K26" s="11" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="L26" s="11" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>
       </c>
-      <c r="L26" s="11" t="inlineStr">
+      <c r="M26" s="11" t="inlineStr">
         <is>
           <t>Reaffirmed all FY2025 guidance.</t>
         </is>
       </c>
-      <c r="M26" s="11" t="inlineStr">
+      <c r="N26" s="11" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-first-quarter-2025-results-and-reaffirms-full-year-guidance-302430212.html</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="58" customHeight="1">
+    <row r="27" ht="60" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>2025-07-17</t>
@@ -2100,26 +2225,31 @@
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>7.5% – 8.0% ex-COVID (6.0% – 7.0% incl.)</t>
-        </is>
-      </c>
-      <c r="K27" s="11" t="inlineStr">
+          <t>7.5% – 8.0% (6.0% – 7.0% incl. COVID)</t>
+        </is>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>Organic, ex-COVID</t>
+        </is>
+      </c>
+      <c r="L27" s="11" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>
       </c>
-      <c r="L27" s="11" t="inlineStr">
+      <c r="M27" s="11" t="inlineStr">
         <is>
           <t>Narrowed adj. EPS range (midpoint unchanged); narrowed organic range.</t>
         </is>
       </c>
-      <c r="M27" s="11" t="inlineStr">
+      <c r="N27" s="11" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-second-quarter-2025-results-302507875.html</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="58" customHeight="1">
+    <row r="28" ht="60" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
           <t>2025-10-15</t>
@@ -2161,26 +2291,31 @@
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>7.5% – 8.0% ex-COVID (6.0% – 7.0% incl.)</t>
-        </is>
-      </c>
-      <c r="K28" s="11" t="inlineStr">
+          <t>7.5% – 8.0% (6.0% – 7.0% incl. COVID)</t>
+        </is>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>Organic, ex-COVID</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>
       </c>
-      <c r="L28" s="11" t="inlineStr">
+      <c r="M28" s="11" t="inlineStr">
         <is>
           <t>Reaffirmed midpoint, narrowed adj. EPS range; reaffirmed organic.</t>
         </is>
       </c>
-      <c r="M28" s="11" t="inlineStr">
+      <c r="N28" s="11" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-third-quarter-2025-results-and-reaffirms-full-year-guidance-302584746.html</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="58" customHeight="1">
+    <row r="29" ht="60" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>2026-01-22</t>
@@ -2225,23 +2360,28 @@
           <t>6.5% – 7.5%</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>Initial FY2026 outlook; ~10% EPS growth at midpoint. Announced acquisition of Exact Sciences.</t>
-        </is>
-      </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
+          <t>Initial FY2026 outlook; ~10% EPS growth at midpoint. Announced acquisition of Exact Sciences (not yet closed at guide).</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-fourth-quarter-and-full-year-2025-results-issues-2026-financial-outlook-302668032.html</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="58" customHeight="1">
+    <row r="30" ht="60" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>2026-04-16</t>
@@ -2283,20 +2423,25 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>6.5% – 7.5% (comparable basis)</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
+          <t>6.5% – 7.5%</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>Comparable (adj. for M&amp;A &amp; FX)</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>EPS lowered to reflect ~$0.20 dilution from Exact Sciences (closed Mar 23, 2026); top-line range maintained, now stated on a 'comparable' basis. Not an operational guide-down.</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/abbott-reports-first-quarter-2026-results-updates-guidance-to-reflect-acquisition-of-exact-sciences-302744652.html</t>
         </is>
@@ -2304,8 +2449,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2317,7 +2462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2326,8 +2471,9 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2340,7 +2486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Read across each block to see how the outlook for a given fiscal year changed quarter to quarter.</t>
+          <t>Read across each block to see how the outlook for a given fiscal year changed quarter to quarter. Sales-growth columns show the headline figure and the basis it was measured on.</t>
         </is>
       </c>
     </row>
@@ -2377,27 +2523,32 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>Sales Growth Guidance</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Sales Growth Basis</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>GAAP EPS Guidance</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Organic / Comparable Sales Growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>FY2020</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Q4 2019</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>2020-01-22</t>
         </is>
@@ -2407,940 +2558,1070 @@
           <t>Initial</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>$3.55 – $3.65</t>
         </is>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="20" t="n">
         <v>3.6</v>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
+          <t>7.0% – 8.0%</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
           <t>$2.35 – $2.45</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>7.0% – 8.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="20" t="n"/>
-      <c r="B6" s="17" t="inlineStr">
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Q1 2020</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>2020-04-16</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Withdrawn</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>Withdrawn / suspended</t>
         </is>
       </c>
-      <c r="F6" s="17" t="n"/>
+      <c r="F6" s="18" t="n"/>
       <c r="G6" s="18" t="inlineStr">
         <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
           <t>Withdrawn / suspended</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="20" t="n"/>
-      <c r="B7" s="17" t="inlineStr">
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Q2 2020</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>2020-07-16</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Reinstated (floor)</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>At least $3.25</t>
         </is>
       </c>
-      <c r="F7" s="17" t="n"/>
+      <c r="F7" s="18" t="n"/>
       <c r="G7" s="18" t="inlineStr">
         <is>
+          <t>Not provided (EPS floor only)</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
           <t>At least $2.00</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="22" t="n"/>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2020</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>2020-10-21</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Raised</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>At least $3.55</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Not provided (EPS floor only)</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>At least $2.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Q4 2020</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>2021-01-27</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="inlineStr">
+        <is>
+          <t>At least $5.00</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>~Double-digit (qualitative; no % issued)</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="I9" s="25" t="inlineStr">
+        <is>
+          <t>At least $3.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="21" t="n"/>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Q1 2021</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>2021-04-20</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Maintained</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>At least $5.00</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="inlineStr">
         <is>
           <t>Not provided (qualitative)</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="21" t="n"/>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Q3 2020</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>2020-10-21</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Not quantified</t>
+        </is>
+      </c>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>At least $3.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="21" t="n"/>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Q2 2021</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>2021-07-22</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Lowered</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>$4.30 – $4.50</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I11" s="25" t="inlineStr">
+        <is>
+          <t>$2.75 – $2.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="22" t="n"/>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Q3 2021</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>2021-10-20</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>At least $3.55</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>At least $2.35</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
-        <is>
-          <t>FY2021</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>Q4 2020</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>2021-01-27</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>$5.00 – $5.10</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I12" s="25" t="inlineStr">
+        <is>
+          <t>$3.55 – $3.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Q4 2021</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>2022-01-26</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Initial</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>At least $5.00</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="n"/>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>At least $3.74</t>
-        </is>
-      </c>
-      <c r="H9" s="24" t="inlineStr">
-        <is>
-          <t>Double-digit (qualitative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>Q1 2021</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>2021-04-20</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>At least $4.70</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>High single digits</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I13" s="28" t="inlineStr">
+        <is>
+          <t>At least $3.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="21" t="n"/>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Q1 2022</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>2022-04-20</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Maintained</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>At least $5.00</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="n"/>
-      <c r="G10" s="24" t="inlineStr">
-        <is>
-          <t>At least $3.74</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>Q2 2021</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>2021-07-22</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>Lowered</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>At least $4.70</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>High single digits</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I14" s="28" t="inlineStr">
+        <is>
+          <t>At least $3.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Q2 2022</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>2022-07-20</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Raised</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>At least $4.90</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>At least $3.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="22" t="n"/>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Q3 2022</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>2022-10-19</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Raised</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>$5.17 – $5.23</t>
+        </is>
+      </c>
+      <c r="F16" s="29" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I16" s="28" t="inlineStr">
+        <is>
+          <t>$3.75 – $3.81</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Q4 2022</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>2023-01-25</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="E17" s="31" t="inlineStr">
         <is>
           <t>$4.30 – $4.50</t>
         </is>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F17" s="32" t="n">
         <v>4.4</v>
       </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>$2.75 – $2.95</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="21" t="n"/>
-      <c r="B12" s="23" t="inlineStr">
-        <is>
-          <t>Q3 2021</t>
-        </is>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>2021-10-20</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>High single digits</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I17" s="31" t="inlineStr">
+        <is>
+          <t>$3.05 – $3.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="21" t="n"/>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Q1 2023</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>2023-04-19</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Maintained</t>
+        </is>
+      </c>
+      <c r="E18" s="31" t="inlineStr">
+        <is>
+          <t>$4.30 – $4.50</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>≈High single digits (raised outlook)</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I18" s="31" t="inlineStr">
+        <is>
+          <t>$3.05 – $3.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="21" t="n"/>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Q2 2023</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>2023-07-20</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Maintained</t>
+        </is>
+      </c>
+      <c r="E19" s="31" t="inlineStr">
+        <is>
+          <t>$4.30 – $4.50</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I19" s="31" t="inlineStr">
+        <is>
+          <t>$3.02 – $3.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="22" t="n"/>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Q3 2023</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>2023-10-18</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Narrowed (midpoint raised)</t>
+        </is>
+      </c>
+      <c r="E20" s="31" t="inlineStr">
+        <is>
+          <t>$4.42 – $4.46</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>Low double digits</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing</t>
+        </is>
+      </c>
+      <c r="I20" s="31" t="inlineStr">
+        <is>
+          <t>$3.14 – $3.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2023</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>2024-01-24</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>$4.50 – $4.70</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>8.0% – 10.0%</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>$3.20 – $3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="21" t="n"/>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2024</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>2024-04-17</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Raised midpoint</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>$4.55 – $4.70</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="n">
+        <v>4.625</v>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>8.5% – 10.0%</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>$3.25 – $3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2024</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>2024-07-18</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Raised</t>
         </is>
       </c>
-      <c r="E12" s="24" t="inlineStr">
-        <is>
-          <t>$5.00 – $5.10</t>
-        </is>
-      </c>
-      <c r="F12" s="25" t="n">
-        <v>5.05</v>
-      </c>
-      <c r="G12" s="24" t="inlineStr">
-        <is>
-          <t>$3.55 – $3.65</t>
-        </is>
-      </c>
-      <c r="H12" s="24" t="inlineStr">
-        <is>
-          <t>Not provided (qualitative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>FY2022</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Q4 2021</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>2022-01-26</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>$4.61 – $4.71</t>
+        </is>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>9.5% – 10.0%</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>$3.30 – $3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="22" t="n"/>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2024</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>2024-10-16</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Raised midpoint / narrowed</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>$4.64 – $4.70</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>9.5% – 10.0%</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial)</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
+        <is>
+          <t>$3.34 – $3.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Q4 2024</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>2025-01-22</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Initial</t>
         </is>
       </c>
-      <c r="E13" s="27" t="inlineStr">
-        <is>
-          <t>At least $4.70</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="27" t="inlineStr">
-        <is>
-          <t>At least $3.43</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="inlineStr">
-        <is>
-          <t>Not stated as single number</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Q1 2022</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>2022-04-20</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Maintained</t>
-        </is>
-      </c>
-      <c r="E14" s="27" t="inlineStr">
-        <is>
-          <t>At least $4.70</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="27" t="inlineStr">
-        <is>
-          <t>At least $3.35</t>
-        </is>
-      </c>
-      <c r="H14" s="27" t="inlineStr">
-        <is>
-          <t>Not stated as single number</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Q2 2022</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>2022-07-20</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Raised</t>
-        </is>
-      </c>
-      <c r="E15" s="27" t="inlineStr">
-        <is>
-          <t>At least $4.90</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="27" t="inlineStr">
-        <is>
-          <t>At least $3.50</t>
-        </is>
-      </c>
-      <c r="H15" s="27" t="inlineStr">
-        <is>
-          <t>Low double digits (base business)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="21" t="n"/>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Q3 2022</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>2022-10-19</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>Raised</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="inlineStr">
-        <is>
-          <t>$5.17 – $5.23</t>
-        </is>
-      </c>
-      <c r="F16" s="28" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G16" s="27" t="inlineStr">
-        <is>
-          <t>$3.75 – $3.81</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="inlineStr">
-        <is>
-          <t>Double-digit base business</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
-        <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Q4 2022</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>2023-01-25</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="E25" s="25" t="inlineStr">
+        <is>
+          <t>$5.05 – $5.25</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>7.5% – 8.5%</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="I25" s="25" t="inlineStr">
+        <is>
+          <t>Not provided (discontinued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Q1 2025</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>2025-04-16</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Reaffirmed</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>$5.05 – $5.25</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="G26" s="24" t="inlineStr">
+        <is>
+          <t>7.5% – 8.5%</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>Not provided (discontinued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="21" t="n"/>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Q2 2025</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>2025-07-17</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Narrowed</t>
+        </is>
+      </c>
+      <c r="E27" s="25" t="inlineStr">
+        <is>
+          <t>$5.10 – $5.20</t>
+        </is>
+      </c>
+      <c r="F27" s="26" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>7.5% – 8.0% (6.0% – 7.0% incl. COVID)</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>Organic, ex-COVID</t>
+        </is>
+      </c>
+      <c r="I27" s="25" t="inlineStr">
+        <is>
+          <t>Not provided (discontinued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="22" t="n"/>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Q3 2025</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Reaffirmed / narrowed</t>
+        </is>
+      </c>
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>$5.12 – $5.18</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>7.5% – 8.0% (6.0% – 7.0% incl. COVID)</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Organic, ex-COVID</t>
+        </is>
+      </c>
+      <c r="I28" s="25" t="inlineStr">
+        <is>
+          <t>Not provided (discontinued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Initial</t>
         </is>
       </c>
-      <c r="E17" s="30" t="inlineStr">
-        <is>
-          <t>$4.30 – $4.50</t>
-        </is>
-      </c>
-      <c r="F17" s="31" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G17" s="30" t="inlineStr">
-        <is>
-          <t>$3.05 – $3.25</t>
-        </is>
-      </c>
-      <c r="H17" s="30" t="inlineStr">
-        <is>
-          <t>High-single digits (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Q1 2023</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>2023-04-19</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Maintained</t>
-        </is>
-      </c>
-      <c r="E18" s="30" t="inlineStr">
-        <is>
-          <t>$4.30 – $4.50</t>
-        </is>
-      </c>
-      <c r="F18" s="31" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G18" s="30" t="inlineStr">
-        <is>
-          <t>$3.05 – $3.25</t>
-        </is>
-      </c>
-      <c r="H18" s="30" t="inlineStr">
-        <is>
-          <t>At least high-single digits (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>Q2 2023</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>2023-07-20</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>Maintained</t>
-        </is>
-      </c>
-      <c r="E19" s="30" t="inlineStr">
-        <is>
-          <t>$4.30 – $4.50</t>
-        </is>
-      </c>
-      <c r="F19" s="31" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G19" s="30" t="inlineStr">
-        <is>
-          <t>$3.02 – $3.22</t>
-        </is>
-      </c>
-      <c r="H19" s="30" t="inlineStr">
-        <is>
-          <t>Low double digits (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="21" t="n"/>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Q3 2023</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>2023-10-18</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Narrowed (midpoint raised)</t>
-        </is>
-      </c>
-      <c r="E20" s="30" t="inlineStr">
-        <is>
-          <t>$4.42 – $4.46</t>
-        </is>
-      </c>
-      <c r="F20" s="31" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="G20" s="30" t="inlineStr">
-        <is>
-          <t>$3.14 – $3.18</t>
-        </is>
-      </c>
-      <c r="H20" s="30" t="inlineStr">
-        <is>
-          <t>Low double digits (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Q4 2023</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>2024-01-24</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Initial</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>$4.50 – $4.70</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G21" s="18" t="inlineStr">
-        <is>
-          <t>$3.20 – $3.40</t>
-        </is>
-      </c>
-      <c r="H21" s="18" t="inlineStr">
-        <is>
-          <t>8.0% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="20" t="n"/>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>Q1 2024</t>
-        </is>
-      </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>2024-04-17</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>Raised midpoint</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>$4.55 – $4.70</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="n">
-        <v>4.625</v>
-      </c>
-      <c r="G22" s="18" t="inlineStr">
-        <is>
-          <t>$3.25 – $3.40</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>8.5% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>Q2 2024</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>2024-07-18</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>Raised</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>$4.61 – $4.71</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="n">
-        <v>4.66</v>
-      </c>
-      <c r="G23" s="18" t="inlineStr">
-        <is>
-          <t>$3.30 – $3.40</t>
-        </is>
-      </c>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>9.5% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="21" t="n"/>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>Q3 2024</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>2024-10-16</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>Raised midpoint / narrowed</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>$4.64 – $4.70</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="G24" s="18" t="inlineStr">
-        <is>
-          <t>$3.34 – $3.40</t>
-        </is>
-      </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>9.5% – 10.0% (ex-COVID)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="22" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>Q4 2024</t>
-        </is>
-      </c>
-      <c r="C25" s="23" t="inlineStr">
-        <is>
-          <t>2025-01-22</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Initial</t>
-        </is>
-      </c>
-      <c r="E25" s="24" t="inlineStr">
-        <is>
-          <t>$5.05 – $5.25</t>
-        </is>
-      </c>
-      <c r="F25" s="25" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="G25" s="24" t="inlineStr">
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>$5.55 – $5.80</t>
+        </is>
+      </c>
+      <c r="F29" s="29" t="n">
+        <v>5.675</v>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>6.5% – 7.5%</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Total-company organic</t>
+        </is>
+      </c>
+      <c r="I29" s="28" t="inlineStr">
         <is>
           <t>Not provided (discontinued)</t>
         </is>
       </c>
-      <c r="H25" s="24" t="inlineStr">
-        <is>
-          <t>7.5% – 8.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>Q1 2025</t>
-        </is>
-      </c>
-      <c r="C26" s="23" t="inlineStr">
-        <is>
-          <t>2025-04-16</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Reaffirmed</t>
-        </is>
-      </c>
-      <c r="E26" s="24" t="inlineStr">
-        <is>
-          <t>$5.05 – $5.25</t>
-        </is>
-      </c>
-      <c r="F26" s="25" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="G26" s="24" t="inlineStr">
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="22" t="n"/>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>Lowered (acquisition dilution)</t>
+        </is>
+      </c>
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>$5.38 – $5.58</t>
+        </is>
+      </c>
+      <c r="F30" s="29" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>6.5% – 7.5%</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Comparable (adj. for M&amp;A &amp; FX)</t>
+        </is>
+      </c>
+      <c r="I30" s="28" t="inlineStr">
         <is>
           <t>Not provided (discontinued)</t>
-        </is>
-      </c>
-      <c r="H26" s="24" t="inlineStr">
-        <is>
-          <t>7.5% – 8.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="20" t="n"/>
-      <c r="B27" s="23" t="inlineStr">
-        <is>
-          <t>Q2 2025</t>
-        </is>
-      </c>
-      <c r="C27" s="23" t="inlineStr">
-        <is>
-          <t>2025-07-17</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Narrowed</t>
-        </is>
-      </c>
-      <c r="E27" s="24" t="inlineStr">
-        <is>
-          <t>$5.10 – $5.20</t>
-        </is>
-      </c>
-      <c r="F27" s="25" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="G27" s="24" t="inlineStr">
-        <is>
-          <t>Not provided (discontinued)</t>
-        </is>
-      </c>
-      <c r="H27" s="24" t="inlineStr">
-        <is>
-          <t>7.5% – 8.0% ex-COVID (6.0% – 7.0% incl.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="21" t="n"/>
-      <c r="B28" s="23" t="inlineStr">
-        <is>
-          <t>Q3 2025</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Reaffirmed / narrowed</t>
-        </is>
-      </c>
-      <c r="E28" s="24" t="inlineStr">
-        <is>
-          <t>$5.12 – $5.18</t>
-        </is>
-      </c>
-      <c r="F28" s="25" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="G28" s="24" t="inlineStr">
-        <is>
-          <t>Not provided (discontinued)</t>
-        </is>
-      </c>
-      <c r="H28" s="24" t="inlineStr">
-        <is>
-          <t>7.5% – 8.0% ex-COVID (6.0% – 7.0% incl.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="26" t="inlineStr">
-        <is>
-          <t>FY2026</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Q4 2025</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Initial</t>
-        </is>
-      </c>
-      <c r="E29" s="27" t="inlineStr">
-        <is>
-          <t>$5.55 – $5.80</t>
-        </is>
-      </c>
-      <c r="F29" s="28" t="n">
-        <v>5.675</v>
-      </c>
-      <c r="G29" s="27" t="inlineStr">
-        <is>
-          <t>Not provided (discontinued)</t>
-        </is>
-      </c>
-      <c r="H29" s="27" t="inlineStr">
-        <is>
-          <t>6.5% – 7.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="21" t="n"/>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Q1 2026</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
-        <is>
-          <t>Lowered (acquisition dilution)</t>
-        </is>
-      </c>
-      <c r="E30" s="27" t="inlineStr">
-        <is>
-          <t>$5.38 – $5.58</t>
-        </is>
-      </c>
-      <c r="F30" s="28" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="G30" s="27" t="inlineStr">
-        <is>
-          <t>Not provided (discontinued)</t>
-        </is>
-      </c>
-      <c r="H30" s="27" t="inlineStr">
-        <is>
-          <t>6.5% – 7.5% (comparable basis)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A17:A20"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A21:A24"/>
     <mergeCell ref="A5:A8"/>
@@ -3356,7 +3637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3371,278 +3652,400 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="32" t="inlineStr"/>
+      <c r="B2" s="33" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="B3" s="33" t="inlineStr">
+      <c r="B3" s="34" t="inlineStr">
         <is>
           <t>WHAT THIS SHOWS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>Each row is the full-year guidance Abbott provided at a given quarterly earnings report. 'Action' flags whether that update</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="32" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>set initial guidance or raised / lowered / maintained / narrowed / withdrew it versus the prior update for the same fiscal year.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="32" t="inlineStr"/>
+      <c r="B6" s="33" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="B7" s="33" t="inlineStr">
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>READING THE SALES-GROWTH COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>Abbott's headline top-line metric changed with the COVID cycle, so 'Sales Growth Basis' tells you what each figure measures:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>• Total-company organic — a clean organic % for the whole company (FY2020 initial; FY2025; FY2026 initial).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>• Base business, ex-COVID testing — Abbott's preferred metric during 2021-2023; it strips out volatile COVID-test sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  In those years Abbott usually gave a DESCRIPTOR ('high single digits' / 'low double digits') rather than a numeric range,</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and put hard numbers only on EPS and on the COVID-testing-sales dollar forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>• Organic (COVID immaterial) — from FY2024, with COVID negligible, Abbott returned to a single organic range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>• Comparable (adj. for M&amp;A &amp; FX) — FY2026 Q1 relabeling that neutralizes the Exact Sciences acquisition and FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>• Not quantified — no sales-growth figure was issued (e.g., the 2020 EPS-floor-only reinstatements; FY2021 setting).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="33" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="34" t="inlineStr">
+        <is>
+          <t>NOTABLE SALES-GROWTH PATTERN (2022 &amp; 2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>Both years followed the same arc: base-business organic set at 'high single digits', raised to 'low double digits' by mid-year</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>as base-business strength offset declining COVID-testing revenue — while adjusted EPS was held roughly flat each time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="33" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="34" t="inlineStr">
         <is>
           <t>KEY STRUCTURAL POINTS</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="32" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>• 2020-2022 were dominated by COVID-19 testing. Abbott withdrew FY2020 guidance entirely in Apr 2020, reinstated it as an</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  'at least' floor mid-year, then raised it. FY2021-2022 guidance swung sharply with COVID-test demand (e.g., FY2021 was</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  cut in Q2 2021 as testing fell, then raised in Q3 2021 during the Delta wave).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="32" t="inlineStr">
-        <is>
-          <t>• 'At least $X' entries are floor guidance (common in 2020-2022); numeric Low/High columns leave the High blank for these.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="32" t="inlineStr">
-        <is>
-          <t>• GAAP EPS guidance was discontinued starting with the FY2025 outlook (Jan 2025): Abbott states it cannot reliably forecast</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  special items (restructuring, impairments, acquisition charges). 'Not provided (discontinued)' reflects that policy change,</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  not missing data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>• Organic sales-growth guidance was given as an explicit % range only at the initial FY2020 outlook and from FY2024 onward.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  In 2020-2023 Abbott mostly guided on EPS and described sales qualitatively (e.g., 'double-digit base business ex-COVID').</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  From FY2024 the headline organic figure excludes COVID testing; FY2025 gave both ex-COVID and all-in ranges.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="32" t="inlineStr">
-        <is>
-          <t>• Q1 2026: adjusted EPS was lowered purely to reflect ~$0.20 of dilution from the Exact Sciences acquisition (closed Mar 23,</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026); the top-line growth range was maintained and restated on a 'comparable' basis. This is not an operational guide-down.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="32" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>DATA CONFIDENCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="32" t="inlineStr">
-        <is>
-          <t>• Adjusted-EPS figures are the highest-confidence numbers and were corroborated across at least two sources per quarter.</t>
-        </is>
-      </c>
-    </row>
     <row r="23">
-      <c r="B23" s="32" t="inlineStr">
-        <is>
-          <t>• A few items carry minor uncertainty: the initial FY2022 GAAP floor (cited as ~$3.43 vs $3.40) and the exact restated</t>
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  'at least' EPS floor mid-year, then raised it. FY2021-2022 swung sharply with COVID-test demand (FY2021 EPS was cut in</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  COVID-testing-sales assumptions at Q3 2022 / Q3 2023 (only the quarter's actual COVID sales were confirmed).</t>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q2 2021 as testing fell, then raised in Q3 2021 during the Delta wave).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="32" t="inlineStr"/>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>• 'At least $X' EPS entries are floor guidance (common 2020-2022); numeric Low/High columns leave the High blank for these.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="33" t="inlineStr">
         <is>
-          <t>REPORTING-DATE NOTES</t>
+          <t>• GAAP EPS guidance was discontinued starting with the FY2025 outlook (Jan 2025): Abbott states it cannot reliably forecast</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="32" t="inlineStr">
-        <is>
-          <t>• FY2021 initial guidance was issued Jan 27, 2021 (Q4 2020 report). FY2021 Q2 cut was first signaled off-cycle in mid-June 2021,</t>
+      <c r="B27" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  special items (restructuring, impairments, acquisition charges). 'Not provided (discontinued)' reflects that policy change.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  then formalized as the $4.30-$4.50 range at the Jul 22, 2021 report.</t>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>• FY2021 had the least numeric sales guidance: at the Jan 2021 setting Abbott issued NO full-year sales-growth %; the first</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="32" t="inlineStr"/>
+      <c r="B29" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  numeric base-business label ('low double digits') came at an off-cycle update on Jun 1, 2021.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>PRIMARY SOURCES</t>
+          <t>• Q1 2026: adjusted EPS was lowered purely to reflect ~$0.20 of dilution from the Exact Sciences acquisition (closed Mar 23,</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="32" t="inlineStr">
-        <is>
-          <t>Abbott investor news (abbott.mediaroom.com) and PR Newswire press releases, plus the corresponding SEC 8-K exhibit 99.1 for</t>
+      <c r="B31" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2026); the top-line growth range was maintained and restated on a 'comparable' basis. Not an operational guide-down.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="32" t="inlineStr">
-        <is>
-          <t>each quarter. Per-row source links are in the 'Source' column of the Guidance Timeline sheet. Secondary cross-checks included</t>
-        </is>
-      </c>
+      <c r="B32" s="33" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="B33" s="32" t="inlineStr">
-        <is>
-          <t>Nasdaq, StockTitan, RTTNews, MedTech Dive, 360Dx and Investing.com.</t>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>DATA CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="32" t="inlineStr"/>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>• Adjusted-EPS figures are the highest-confidence numbers and were corroborated across at least two sources per quarter.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="B35" s="32" t="inlineStr">
-        <is>
-          <t>Compiled 2026-06-05. Figures are guidance as issued at the time of each report, not actuals. For an auditable record, confirm</t>
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>• Minor uncertainty: the initial FY2022 GAAP floor (cited as ~$3.43 vs $3.40); the exact COVID-testing-sales assumption at</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="32" t="inlineStr">
-        <is>
-          <t>each figure against the linked SEC 8-K / press release.</t>
-        </is>
-      </c>
+      <c r="B36" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q3 2022 (~$7.8B) and the implied FY2023 figure at Q3 2023; and the precise wording of the Q1 2023 base-business descriptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ('high single digits' vs 'at least high single digits').</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="33" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="B39" s="34" t="inlineStr">
         <is>
+          <t>PRIMARY SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>Abbott investor news (abbott.mediaroom.com) and PR Newswire press releases, plus the corresponding SEC 8-K exhibit 99.1 for</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="33" t="inlineStr">
+        <is>
+          <t>each quarter. Per-row source links are in the 'Source' column of the Guidance Timeline sheet. Secondary cross-checks included</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>Nasdaq, StockTitan, RTTNews, MedTech Dive, 360Dx, Motley Fool / Seeking Alpha transcripts and Investing.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="33" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="33" t="inlineStr">
+        <is>
+          <t>Compiled 2026-06-05. Figures are guidance as issued at the time of each report, not actuals. For an auditable record, confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="33" t="inlineStr">
+        <is>
+          <t>each figure against the linked SEC 8-K / press release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="35" t="inlineStr">
+        <is>
           <t>ACTION COLOR LEGEND</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="35" t="n"/>
-      <c r="B40" s="36" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="36" t="n"/>
+      <c r="B49" s="37" t="inlineStr">
         <is>
           <t>Initial — Initial outlook for a fiscal year</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="37" t="n"/>
-      <c r="B41" s="36" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="38" t="n"/>
+      <c r="B50" s="37" t="inlineStr">
         <is>
           <t>Raised — Guidance raised vs prior update</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="38" t="n"/>
-      <c r="B42" s="36" t="inlineStr">
-        <is>
-          <t>Maintained / Reaffirmed / Narrowed — Held or tightened around the same midpoint</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="39" t="n"/>
-      <c r="B43" s="36" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="39" t="n"/>
+      <c r="B51" s="37" t="inlineStr">
+        <is>
+          <t>Maintained — Held or reaffirmed around the same level</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="39" t="n"/>
+      <c r="B52" s="37" t="inlineStr">
+        <is>
+          <t>Narrowed (midpoint raised) — Range tightened, midpoint up</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="40" t="n"/>
+      <c r="B53" s="37" t="inlineStr">
         <is>
           <t>Reinstated (floor) — Guidance restored as an 'at least' floor</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="40" t="n"/>
-      <c r="B44" s="36" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="41" t="n"/>
+      <c r="B54" s="37" t="inlineStr">
         <is>
           <t>Lowered — Guidance reduced vs prior update</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="41" t="n"/>
-      <c r="B45" s="36" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="42" t="n"/>
+      <c r="B55" s="37" t="inlineStr">
         <is>
           <t>Withdrawn — Guidance suspended</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="35" t="inlineStr">
+        <is>
+          <t>SALES GROWTH BASIS COLOR LEGEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="38" t="n"/>
+      <c r="B58" s="37" t="inlineStr">
+        <is>
+          <t>Total-company organic — Clean organic % for the whole company</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="38" t="n"/>
+      <c r="B59" s="37" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial) — Single organic range, COVID negligible (FY2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="43" t="n"/>
+      <c r="B60" s="37" t="inlineStr">
+        <is>
+          <t>Organic, ex-COVID — Organic excluding residual COVID testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="39" t="n"/>
+      <c r="B61" s="37" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing — Underlying growth ex-COVID (often a descriptor, 2021-2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="36" t="n"/>
+      <c r="B62" s="37" t="inlineStr">
+        <is>
+          <t>Comparable (adj. for M&amp;A &amp; FX) — Adjusted for the Exact Sciences acquisition &amp; FX (FY2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="42" t="n"/>
+      <c r="B63" s="37" t="inlineStr">
+        <is>
+          <t>Not quantified — No sales-growth figure issued</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Trends tab with EPS and organic-growth guidance trajectory charts
- New Trends sheet with two line charts: adjusted-EPS guidance midpoint
  (floor used for 'at least $X' guidance) and organic-growth midpoint
  (numeric quarters only) across all 26 reports
- Underlying chart data block kept on the same sheet for transparency

https://claude.ai/code/session_01EKrf5kyJ9fDoQd1dRoC1pG
</commit_message>
<xml_diff>
--- a/Abbott_Guidance_By_Quarter_2020-2026.xlsx
+++ b/Abbott_Guidance_By_Quarter_2020-2026.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Guidance Timeline" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="By Fiscal Year" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Notes &amp; Sources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Trends" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +62,11 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="14">
@@ -190,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -295,6 +301,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -369,6 +376,294 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Abbott adjusted EPS guidance over time</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trends'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trends'!$A$5:$A$30</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trends'!$B$5:$B$30</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Earnings report</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Adjusted EPS ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Abbott organic / comparable sales-growth guidance midpoint (where numeric)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trends'!C4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trends'!$A$5:$A$30</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trends'!$C$5:$C$30</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Earnings report</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Organic growth midpoint (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4052,4 +4347,349 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Guidance Trajectory — adjusted EPS and organic sales-growth midpoints over time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EPS line uses the guidance midpoint, or the floor for 'at least $X' guidance. Organic line shows the midpoint only for quarters where Abbott gave a numeric range (FY2020 initial, FY2024 onward).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>Adj. EPS guide point ($)</t>
+        </is>
+      </c>
+      <c r="C4" s="44" t="inlineStr">
+        <is>
+          <t>Organic growth midpoint (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q4 2019 (2020)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Q1 2020 (2020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Q2 2020 (2020)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Q3 2020 (2020)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.55</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Q4 2020 (2021)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Q1 2021 (2021)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q2 2021 (2021)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Q3 2021 (2021)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Q4 2021 (2022)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q1 2022 (2022)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q2 2022 (2022)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q3 2022 (2022)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Q4 2022 (2023)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q1 2023 (2023)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Q2 2023 (2023)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Q3 2023 (2023)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4.44</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Q4 2023 (2024)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Q1 2024 (2024)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4.625</v>
+      </c>
+      <c r="C22" t="n">
+        <v>9.25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Q2 2024 (2024)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="C23" t="n">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Q3 2024 (2024)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="C24" t="n">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Q4 2024 (2025)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="C25" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q1 2025 (2025)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Q2 2025 (2025)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="C27" t="n">
+        <v>7.75</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Q3 2025 (2025)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7.75</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Q4 2025 (2026)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5.675</v>
+      </c>
+      <c r="C29" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Q1 2026 (2026)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="C30" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Growth to Guidance calculator tab
New formula-driven tab quantifying how much growth is still needed to
reach guidance and consensus:

- Live FY2026 calculators (adjusted EPS and comparable sales): given
  Q1'26 actuals, compute the Q2-Q4 growth required to hit the low/mid/high
  of guidance and a user-entered consensus
- Per-fiscal-year backtest (2020-2026): prior-year base, actual results,
  guidance-implied vs actual EPS/sales growth, with a yellow consensus
  input column per year and auto-computed actual-vs-consensus gap
- Built on Abbott reported actuals (net sales & adjusted EPS 2019-2025,
  FY2025 quarterly EPS, Q1'26 YTD); consensus cells left blank to populate
- Notes tab documents the actuals, sources, and the sales-weighting caveat

https://claude.ai/code/session_01EKrf5kyJ9fDoQd1dRoC1pG
</commit_message>
<xml_diff>
--- a/Abbott_Guidance_By_Quarter_2020-2026.xlsx
+++ b/Abbott_Guidance_By_Quarter_2020-2026.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Guidance Timeline" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="By Fiscal Year" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes &amp; Sources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Growth to Guidance" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Trends" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Notes &amp; Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +55,34 @@
       <sz val="10"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F3864"/>
@@ -69,7 +99,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -136,8 +166,18 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F7FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -192,11 +232,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B4C6E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B4C6E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4C6E7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -286,13 +359,63 @@
     <xf numFmtId="164" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -301,7 +424,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3932,419 +4054,811 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Notes, Methodology &amp; Sources</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Growth Needed to Reach Guidance &amp; Consensus</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="33" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="34" t="inlineStr">
-        <is>
-          <t>WHAT THIS SHOWS</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Yellow cells = inputs you populate (consensus). White/blue cells compute automatically in Excel. FY2026 is the live year (Q1 reported); the lower table backtests every year and accepts consensus EPS.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="33" t="inlineStr">
-        <is>
-          <t>Each row is the full-year guidance Abbott provided at a given quarterly earnings report. 'Action' flags whether that update</t>
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>FY2026  ·  Adjusted EPS — growth still needed to reach guidance &amp; consensus</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="33" t="inlineStr">
-        <is>
-          <t>set initial guidance or raised / lowered / maintained / narrowed / withdrew it versus the prior update for the same fiscal year.</t>
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Guidance Low</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Guidance Mid</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Guidance High</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Consensus (input)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="33" t="inlineStr"/>
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Full-year target — adjusted EPS ($)</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="E6" s="37" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t>READING THE SALES-GROWTH COLUMNS</t>
-        </is>
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Prior-year actual — FY2025 ($)</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="C7" s="36">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="D7" s="36">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="E7" s="36">
+        <f>$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>Abbott's headline top-line metric changed with the COVID cycle, so 'Sales Growth Basis' tells you what each figure measures:</t>
-        </is>
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Implied full-year EPS growth vs FY2025</t>
+        </is>
+      </c>
+      <c r="B8" s="38">
+        <f>B6/$B$7-1</f>
+        <v/>
+      </c>
+      <c r="C8" s="38">
+        <f>C6/$B$7-1</f>
+        <v/>
+      </c>
+      <c r="D8" s="38">
+        <f>D6/$B$7-1</f>
+        <v/>
+      </c>
+      <c r="E8" s="38">
+        <f>E6/$B$7-1</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>• Total-company organic — a clean organic % for the whole company (FY2020 initial; FY2025; FY2026 initial).</t>
-        </is>
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>YTD actual — Q1'26 ($)</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C9" s="36">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="D9" s="36">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="E9" s="36">
+        <f>$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>• Base business, ex-COVID testing — Abbott's preferred metric during 2021-2023; it strips out volatile COVID-test sales.</t>
-        </is>
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Prior-year YTD — Q1'25 ($)</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="C10" s="36">
+        <f>$B$10</f>
+        <v/>
+      </c>
+      <c r="D10" s="36">
+        <f>$B$10</f>
+        <v/>
+      </c>
+      <c r="E10" s="36">
+        <f>$B$10</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  In those years Abbott usually gave a DESCRIPTOR ('high single digits' / 'low double digits') rather than a numeric range,</t>
-        </is>
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>YTD growth achieved (Q1'26 vs Q1'25)</t>
+        </is>
+      </c>
+      <c r="B11" s="38">
+        <f>$B$9/$B$10-1</f>
+        <v/>
+      </c>
+      <c r="C11" s="38">
+        <f>$B$9/$B$10-1</f>
+        <v/>
+      </c>
+      <c r="D11" s="38">
+        <f>$B$9/$B$10-1</f>
+        <v/>
+      </c>
+      <c r="E11" s="38">
+        <f>$B$9/$B$10-1</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  and put hard numbers only on EPS and on the COVID-testing-sales dollar forecast.</t>
-        </is>
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>Remaining (Q2–Q4) EPS still needed ($)</t>
+        </is>
+      </c>
+      <c r="B12" s="39">
+        <f>B6-$B$9</f>
+        <v/>
+      </c>
+      <c r="C12" s="39">
+        <f>C6-$B$9</f>
+        <v/>
+      </c>
+      <c r="D12" s="39">
+        <f>D6-$B$9</f>
+        <v/>
+      </c>
+      <c r="E12" s="39">
+        <f>E6-$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>• Organic (COVID immaterial) — from FY2024, with COVID negligible, Abbott returned to a single organic range.</t>
-        </is>
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>Prior-year remaining — Q2–Q4'25 ($)</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="C13" s="36">
+        <f>$B$13</f>
+        <v/>
+      </c>
+      <c r="D13" s="36">
+        <f>$B$13</f>
+        <v/>
+      </c>
+      <c r="E13" s="36">
+        <f>$B$13</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>• Comparable (adj. for M&amp;A &amp; FX) — FY2026 Q1 relabeling that neutralizes the Exact Sciences acquisition and FX.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="33" t="inlineStr">
-        <is>
-          <t>• Not quantified — no sales-growth figure was issued (e.g., the 2020 EPS-floor-only reinstatements; FY2021 setting).</t>
-        </is>
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>Required Q2–Q4 EPS growth to hit target</t>
+        </is>
+      </c>
+      <c r="B14" s="41">
+        <f>B12/$B$13-1</f>
+        <v/>
+      </c>
+      <c r="C14" s="41">
+        <f>C12/$B$13-1</f>
+        <v/>
+      </c>
+      <c r="D14" s="41">
+        <f>D12/$B$13-1</f>
+        <v/>
+      </c>
+      <c r="E14" s="41">
+        <f>E12/$B$13-1</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="33" t="inlineStr"/>
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>FY2026  ·  Sales (comparable growth) — growth still needed to reach guidance &amp; consensus</t>
+        </is>
+      </c>
     </row>
     <row r="17">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
       <c r="B17" s="34" t="inlineStr">
         <is>
-          <t>NOTABLE SALES-GROWTH PATTERN (2022 &amp; 2023)</t>
-        </is>
-      </c>
+          <t>Guidance Low</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="inlineStr">
+        <is>
+          <t>Guidance Mid</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>Guidance High</t>
+        </is>
+      </c>
+      <c r="E17" s="34" t="inlineStr">
+        <is>
+          <t>Consensus (input)</t>
+        </is>
+      </c>
+      <c r="G17" s="42" t="inlineStr">
+        <is>
+          <t>Prior-yr sales weights ($M)</t>
+        </is>
+      </c>
+      <c r="H17" s="43" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>Both years followed the same arc: base-business organic set at 'high single digits', raised to 'low double digits' by mid-year</t>
-        </is>
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>Full-year comparable sales-growth target</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="C18" s="44" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D18" s="44" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="E18" s="45" t="n"/>
+      <c r="G18" s="35" t="inlineStr">
+        <is>
+          <t>FY2025 full-year</t>
+        </is>
+      </c>
+      <c r="H18" s="46" t="n">
+        <v>44328</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>as base-business strength offset declining COVID-testing revenue — while adjusted EPS was held roughly flat each time.</t>
-        </is>
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>YTD (Q1'26) comparable growth achieved</t>
+        </is>
+      </c>
+      <c r="B19" s="44" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="C19" s="44">
+        <f>$B$19</f>
+        <v/>
+      </c>
+      <c r="D19" s="44">
+        <f>$B$19</f>
+        <v/>
+      </c>
+      <c r="E19" s="44">
+        <f>$B$19</f>
+        <v/>
+      </c>
+      <c r="G19" s="35" t="inlineStr">
+        <is>
+          <t>Q1'25</t>
+        </is>
+      </c>
+      <c r="H19" s="46" t="n">
+        <v>10358</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="33" t="inlineStr"/>
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>Required Q2–Q4 comparable growth to hit target</t>
+        </is>
+      </c>
+      <c r="B20" s="41">
+        <f>(B18*$H$18-$B$19*$H$19)/$H$20</f>
+        <v/>
+      </c>
+      <c r="C20" s="41">
+        <f>(C18*$H$18-$B$19*$H$19)/$H$20</f>
+        <v/>
+      </c>
+      <c r="D20" s="41">
+        <f>(D18*$H$18-$B$19*$H$19)/$H$20</f>
+        <v/>
+      </c>
+      <c r="E20" s="41">
+        <f>(E18*$H$18-$B$19*$H$19)/$H$20</f>
+        <v/>
+      </c>
+      <c r="G20" s="35" t="inlineStr">
+        <is>
+          <t>Q2–Q4'25</t>
+        </is>
+      </c>
+      <c r="H20" s="46" t="n">
+        <v>33970</v>
+      </c>
     </row>
     <row r="21">
-      <c r="B21" s="34" t="inlineStr">
-        <is>
-          <t>KEY STRUCTURAL POINTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>• 2020-2022 were dominated by COVID-19 testing. Abbott withdrew FY2020 guidance entirely in Apr 2020, reinstated it as an</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  'at least' EPS floor mid-year, then raised it. FY2021-2022 swung sharply with COVID-test demand (FY2021 EPS was cut in</t>
+      <c r="A21" s="47" t="inlineStr">
+        <is>
+          <t>Note: the required-remaining-growth row weights quarters by prior-year reported sales (approximation; Abbott's 'comparable' base also adjusts for the Exact Sciences acquisition &amp; FX). EPS calc above is exact (uses actual quarterly EPS).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Q2 2021 as testing fell, then raised in Q3 2021 during the Delta wave).</t>
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>All fiscal years  ·  Guidance-implied growth vs actual results (enter consensus in the yellow column)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>• 'At least $X' EPS entries are floor guidance (common 2020-2022); numeric Low/High columns leave the High blank for these.</t>
+      <c r="A25" s="48" t="inlineStr">
+        <is>
+          <t>FY</t>
+        </is>
+      </c>
+      <c r="B25" s="48" t="inlineStr">
+        <is>
+          <t>Prior-Yr Net Sales ($M)</t>
+        </is>
+      </c>
+      <c r="C25" s="48" t="inlineStr">
+        <is>
+          <t>Actual Net Sales ($M)</t>
+        </is>
+      </c>
+      <c r="D25" s="48" t="inlineStr">
+        <is>
+          <t>Actual Reported Sales Growth</t>
+        </is>
+      </c>
+      <c r="E25" s="48" t="inlineStr">
+        <is>
+          <t>Actual Total Organic %</t>
+        </is>
+      </c>
+      <c r="F25" s="48" t="inlineStr">
+        <is>
+          <t>Actual Base ex-COVID Organic %</t>
+        </is>
+      </c>
+      <c r="G25" s="48" t="inlineStr">
+        <is>
+          <t>Prior-Yr Adj EPS</t>
+        </is>
+      </c>
+      <c r="H25" s="48" t="inlineStr">
+        <is>
+          <t>Actual Adj EPS</t>
+        </is>
+      </c>
+      <c r="I25" s="48" t="inlineStr">
+        <is>
+          <t>Actual EPS Growth</t>
+        </is>
+      </c>
+      <c r="J25" s="48" t="inlineStr">
+        <is>
+          <t>Initial EPS Guidance</t>
+        </is>
+      </c>
+      <c r="K25" s="48" t="inlineStr">
+        <is>
+          <t>Final EPS Guidance</t>
+        </is>
+      </c>
+      <c r="L25" s="48" t="inlineStr">
+        <is>
+          <t>Actual − Initial Guid ($)</t>
+        </is>
+      </c>
+      <c r="M25" s="48" t="inlineStr">
+        <is>
+          <t>Consensus Adj EPS (input)</t>
+        </is>
+      </c>
+      <c r="N25" s="48" t="inlineStr">
+        <is>
+          <t>Actual − Consensus ($)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="33" t="inlineStr">
-        <is>
-          <t>• GAAP EPS guidance was discontinued starting with the FY2025 outlook (Jan 2025): Abbott states it cannot reliably forecast</t>
-        </is>
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="B26" s="46" t="n">
+        <v>31904</v>
+      </c>
+      <c r="C26" s="46" t="n">
+        <v>34608</v>
+      </c>
+      <c r="D26" s="38">
+        <f>C26/B26-1</f>
+        <v/>
+      </c>
+      <c r="E26" s="44" t="n"/>
+      <c r="F26" s="44" t="n"/>
+      <c r="G26" s="36" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="H26" s="36" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="I26" s="38">
+        <f>H26/G26-1</f>
+        <v/>
+      </c>
+      <c r="J26" s="36" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="K26" s="36" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="L26" s="39">
+        <f>H26-J26</f>
+        <v/>
+      </c>
+      <c r="M26" s="37" t="n"/>
+      <c r="N26" s="39">
+        <f>IF(AND(H26&lt;&gt;"",M26&lt;&gt;""),H26-M26,"")</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  special items (restructuring, impairments, acquisition charges). 'Not provided (discontinued)' reflects that policy change.</t>
-        </is>
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="B27" s="46" t="n">
+        <v>34608</v>
+      </c>
+      <c r="C27" s="46" t="n">
+        <v>43075</v>
+      </c>
+      <c r="D27" s="38">
+        <f>C27/B27-1</f>
+        <v/>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="G27" s="36" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="H27" s="36" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="I27" s="38">
+        <f>H27/G27-1</f>
+        <v/>
+      </c>
+      <c r="J27" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="K27" s="36" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="L27" s="39">
+        <f>H27-J27</f>
+        <v/>
+      </c>
+      <c r="M27" s="37" t="n"/>
+      <c r="N27" s="39">
+        <f>IF(AND(H27&lt;&gt;"",M27&lt;&gt;""),H27-M27,"")</f>
+        <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="33" t="inlineStr">
-        <is>
-          <t>• FY2021 had the least numeric sales guidance: at the Jan 2021 setting Abbott issued NO full-year sales-growth %; the first</t>
-        </is>
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="B28" s="46" t="n">
+        <v>43075</v>
+      </c>
+      <c r="C28" s="46" t="n">
+        <v>43653</v>
+      </c>
+      <c r="D28" s="38">
+        <f>C28/B28-1</f>
+        <v/>
+      </c>
+      <c r="E28" s="44" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="F28" s="44" t="n"/>
+      <c r="G28" s="36" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="H28" s="36" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="I28" s="38">
+        <f>H28/G28-1</f>
+        <v/>
+      </c>
+      <c r="J28" s="36" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="K28" s="36" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="L28" s="39">
+        <f>H28-J28</f>
+        <v/>
+      </c>
+      <c r="M28" s="37" t="n"/>
+      <c r="N28" s="39">
+        <f>IF(AND(H28&lt;&gt;"",M28&lt;&gt;""),H28-M28,"")</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  numeric base-business label ('low double digits') came at an off-cycle update on Jun 1, 2021.</t>
-        </is>
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="B29" s="46" t="n">
+        <v>43653</v>
+      </c>
+      <c r="C29" s="46" t="n">
+        <v>40109</v>
+      </c>
+      <c r="D29" s="38">
+        <f>C29/B29-1</f>
+        <v/>
+      </c>
+      <c r="E29" s="44" t="n"/>
+      <c r="F29" s="44" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="G29" s="36" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="H29" s="36" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="I29" s="38">
+        <f>H29/G29-1</f>
+        <v/>
+      </c>
+      <c r="J29" s="36" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="K29" s="36" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="L29" s="39">
+        <f>H29-J29</f>
+        <v/>
+      </c>
+      <c r="M29" s="37" t="n"/>
+      <c r="N29" s="39">
+        <f>IF(AND(H29&lt;&gt;"",M29&lt;&gt;""),H29-M29,"")</f>
+        <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="33" t="inlineStr">
-        <is>
-          <t>• Q1 2026: adjusted EPS was lowered purely to reflect ~$0.20 of dilution from the Exact Sciences acquisition (closed Mar 23,</t>
-        </is>
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="B30" s="46" t="n">
+        <v>40109</v>
+      </c>
+      <c r="C30" s="46" t="n">
+        <v>41950</v>
+      </c>
+      <c r="D30" s="38">
+        <f>C30/B30-1</f>
+        <v/>
+      </c>
+      <c r="E30" s="44" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="F30" s="44" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="G30" s="36" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="H30" s="36" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="I30" s="38">
+        <f>H30/G30-1</f>
+        <v/>
+      </c>
+      <c r="J30" s="36" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="K30" s="36" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="L30" s="39">
+        <f>H30-J30</f>
+        <v/>
+      </c>
+      <c r="M30" s="37" t="n"/>
+      <c r="N30" s="39">
+        <f>IF(AND(H30&lt;&gt;"",M30&lt;&gt;""),H30-M30,"")</f>
+        <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2026); the top-line growth range was maintained and restated on a 'comparable' basis. Not an operational guide-down.</t>
-        </is>
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="B31" s="46" t="n">
+        <v>41950</v>
+      </c>
+      <c r="C31" s="46" t="n">
+        <v>44328</v>
+      </c>
+      <c r="D31" s="38">
+        <f>C31/B31-1</f>
+        <v/>
+      </c>
+      <c r="E31" s="44" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="F31" s="44" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="G31" s="36" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="H31" s="36" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="I31" s="38">
+        <f>H31/G31-1</f>
+        <v/>
+      </c>
+      <c r="J31" s="36" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="K31" s="36" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="L31" s="39">
+        <f>H31-J31</f>
+        <v/>
+      </c>
+      <c r="M31" s="37" t="n"/>
+      <c r="N31" s="39">
+        <f>IF(AND(H31&lt;&gt;"",M31&lt;&gt;""),H31-M31,"")</f>
+        <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="33" t="inlineStr"/>
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="B32" s="46" t="n">
+        <v>44328</v>
+      </c>
+      <c r="C32" s="46" t="n"/>
+      <c r="D32" s="38" t="n"/>
+      <c r="E32" s="44" t="n"/>
+      <c r="F32" s="44" t="n"/>
+      <c r="G32" s="36" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="H32" s="36" t="n"/>
+      <c r="I32" s="38" t="n"/>
+      <c r="J32" s="36" t="n">
+        <v>5.675</v>
+      </c>
+      <c r="K32" s="36" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="L32" s="39" t="n"/>
+      <c r="M32" s="37" t="n"/>
+      <c r="N32" s="39">
+        <f>IF(AND(H32&lt;&gt;"",M32&lt;&gt;""),H32-M32,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
-      <c r="B33" s="34" t="inlineStr">
-        <is>
-          <t>DATA CONFIDENCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="33" t="inlineStr">
-        <is>
-          <t>• Adjusted-EPS figures are the highest-confidence numbers and were corroborated across at least two sources per quarter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>• Minor uncertainty: the initial FY2022 GAAP floor (cited as ~$3.43 vs $3.40); the exact COVID-testing-sales assumption at</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Q3 2022 (~$7.8B) and the implied FY2023 figure at Q3 2023; and the precise wording of the Q1 2023 base-business descriptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ('high single digits' vs 'at least high single digits').</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="33" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="34" t="inlineStr">
-        <is>
-          <t>PRIMARY SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="33" t="inlineStr">
-        <is>
-          <t>Abbott investor news (abbott.mediaroom.com) and PR Newswire press releases, plus the corresponding SEC 8-K exhibit 99.1 for</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="33" t="inlineStr">
-        <is>
-          <t>each quarter. Per-row source links are in the 'Source' column of the Guidance Timeline sheet. Secondary cross-checks included</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="33" t="inlineStr">
-        <is>
-          <t>Nasdaq, StockTitan, RTTNews, MedTech Dive, 360Dx, Motley Fool / Seeking Alpha transcripts and Investing.com.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="33" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="B44" s="33" t="inlineStr">
-        <is>
-          <t>Compiled 2026-06-05. Figures are guidance as issued at the time of each report, not actuals. For an auditable record, confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="33" t="inlineStr">
-        <is>
-          <t>each figure against the linked SEC 8-K / press release.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="35" t="inlineStr">
-        <is>
-          <t>ACTION COLOR LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="36" t="n"/>
-      <c r="B49" s="37" t="inlineStr">
-        <is>
-          <t>Initial — Initial outlook for a fiscal year</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="38" t="n"/>
-      <c r="B50" s="37" t="inlineStr">
-        <is>
-          <t>Raised — Guidance raised vs prior update</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="39" t="n"/>
-      <c r="B51" s="37" t="inlineStr">
-        <is>
-          <t>Maintained — Held or reaffirmed around the same level</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="39" t="n"/>
-      <c r="B52" s="37" t="inlineStr">
-        <is>
-          <t>Narrowed (midpoint raised) — Range tightened, midpoint up</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="40" t="n"/>
-      <c r="B53" s="37" t="inlineStr">
-        <is>
-          <t>Reinstated (floor) — Guidance restored as an 'at least' floor</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="41" t="n"/>
-      <c r="B54" s="37" t="inlineStr">
-        <is>
-          <t>Lowered — Guidance reduced vs prior update</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="42" t="n"/>
-      <c r="B55" s="37" t="inlineStr">
-        <is>
-          <t>Withdrawn — Guidance suspended</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="35" t="inlineStr">
-        <is>
-          <t>SALES GROWTH BASIS COLOR LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="38" t="n"/>
-      <c r="B58" s="37" t="inlineStr">
-        <is>
-          <t>Total-company organic — Clean organic % for the whole company</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="38" t="n"/>
-      <c r="B59" s="37" t="inlineStr">
-        <is>
-          <t>Organic (COVID immaterial) — Single organic range, COVID negligible (FY2024)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="43" t="n"/>
-      <c r="B60" s="37" t="inlineStr">
-        <is>
-          <t>Organic, ex-COVID — Organic excluding residual COVID testing</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="39" t="n"/>
-      <c r="B61" s="37" t="inlineStr">
-        <is>
-          <t>Base business, ex-COVID testing — Underlying growth ex-COVID (often a descriptor, 2021-2023)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="36" t="n"/>
-      <c r="B62" s="37" t="inlineStr">
-        <is>
-          <t>Comparable (adj. for M&amp;A &amp; FX) — Adjusted for the Exact Sciences acquisition &amp; FX (FY2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="42" t="n"/>
-      <c r="B63" s="37" t="inlineStr">
-        <is>
-          <t>Not quantified — No sales-growth figure issued</t>
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>FY2026 in progress: YTD Q1'26 comparable sales growth +3.7%, Q1'26 adjusted EPS $1.15 (vs $1.09). Initial EPS guidance $5.55–$5.80 (mid $5.675); current $5.38–$5.58 (mid $5.48) after Exact Sciences dilution.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A33:N33"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4378,17 +4892,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Report</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>Adj. EPS guide point ($)</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="50" t="inlineStr">
         <is>
           <t>Organic growth midpoint (%)</t>
         </is>
@@ -4692,4 +5206,514 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Notes, Methodology &amp; Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="51" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>WHAT THIS SHOWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="51" t="inlineStr">
+        <is>
+          <t>Each row is the full-year guidance Abbott provided at a given quarterly earnings report. 'Action' flags whether that update</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="51" t="inlineStr">
+        <is>
+          <t>set initial guidance or raised / lowered / maintained / narrowed / withdrew it versus the prior update for the same fiscal year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="51" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="52" t="inlineStr">
+        <is>
+          <t>READING THE SALES-GROWTH COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>Abbott's headline top-line metric changed with the COVID cycle, so 'Sales Growth Basis' tells you what each figure measures:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="51" t="inlineStr">
+        <is>
+          <t>• Total-company organic — a clean organic % for the whole company (FY2020 initial; FY2025; FY2026 initial).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="51" t="inlineStr">
+        <is>
+          <t>• Base business, ex-COVID testing — Abbott's preferred metric during 2021-2023; it strips out volatile COVID-test sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  In those years Abbott usually gave a DESCRIPTOR ('high single digits' / 'low double digits') rather than a numeric range,</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and put hard numbers only on EPS and on the COVID-testing-sales dollar forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="51" t="inlineStr">
+        <is>
+          <t>• Organic (COVID immaterial) — from FY2024, with COVID negligible, Abbott returned to a single organic range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="51" t="inlineStr">
+        <is>
+          <t>• Comparable (adj. for M&amp;A &amp; FX) — FY2026 Q1 relabeling that neutralizes the Exact Sciences acquisition and FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="51" t="inlineStr">
+        <is>
+          <t>• Not quantified — no sales-growth figure was issued (e.g., the 2020 EPS-floor-only reinstatements; FY2021 setting).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="51" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="52" t="inlineStr">
+        <is>
+          <t>NOTABLE SALES-GROWTH PATTERN (2022 &amp; 2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="51" t="inlineStr">
+        <is>
+          <t>Both years followed the same arc: base-business organic set at 'high single digits', raised to 'low double digits' by mid-year</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="51" t="inlineStr">
+        <is>
+          <t>as base-business strength offset declining COVID-testing revenue — while adjusted EPS was held roughly flat each time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="51" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="52" t="inlineStr">
+        <is>
+          <t>KEY STRUCTURAL POINTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>• 2020-2022 were dominated by COVID-19 testing. Abbott withdrew FY2020 guidance entirely in Apr 2020, reinstated it as an</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  'at least' EPS floor mid-year, then raised it. FY2021-2022 swung sharply with COVID-test demand (FY2021 EPS was cut in</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q2 2021 as testing fell, then raised in Q3 2021 during the Delta wave).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>• 'At least $X' EPS entries are floor guidance (common 2020-2022); numeric Low/High columns leave the High blank for these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>• GAAP EPS guidance was discontinued starting with the FY2025 outlook (Jan 2025): Abbott states it cannot reliably forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  special items (restructuring, impairments, acquisition charges). 'Not provided (discontinued)' reflects that policy change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="51" t="inlineStr">
+        <is>
+          <t>• FY2021 had the least numeric sales guidance: at the Jan 2021 setting Abbott issued NO full-year sales-growth %; the first</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  numeric base-business label ('low double digits') came at an off-cycle update on Jun 1, 2021.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="51" t="inlineStr">
+        <is>
+          <t>• Q1 2026: adjusted EPS was lowered purely to reflect ~$0.20 of dilution from the Exact Sciences acquisition (closed Mar 23,</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2026); the top-line growth range was maintained and restated on a 'comparable' basis. Not an operational guide-down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="51" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="52" t="inlineStr">
+        <is>
+          <t>DATA CONFIDENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="51" t="inlineStr">
+        <is>
+          <t>• Adjusted-EPS figures are the highest-confidence numbers and were corroborated across at least two sources per quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="51" t="inlineStr">
+        <is>
+          <t>• Minor uncertainty: the initial FY2022 GAAP floor (cited as ~$3.43 vs $3.40); the exact COVID-testing-sales assumption at</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q3 2022 (~$7.8B) and the implied FY2023 figure at Q3 2023; and the precise wording of the Q1 2023 base-business descriptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ('high single digits' vs 'at least high single digits').</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="51" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="52" t="inlineStr">
+        <is>
+          <t>GROWTH TO GUIDANCE TAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="51" t="inlineStr">
+        <is>
+          <t>A calculator showing how much growth is still needed to reach guidance and consensus. Yellow cells are inputs (consensus);</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="51" t="inlineStr">
+        <is>
+          <t>everything else recomputes in Excel. The top blocks track the live FY2026 year: given Q1'26 actuals, they show the Q2-Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="51" t="inlineStr">
+        <is>
+          <t>growth required to land at the low/mid/high of guidance (and at a consensus you enter). The lower table backtests every</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="51" t="inlineStr">
+        <is>
+          <t>fiscal year (guidance-implied growth vs actual results) and accepts a consensus adj. EPS per year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="51" t="inlineStr">
+        <is>
+          <t>Actuals used (Abbott reported): net sales ($M) 2019: 31,904; 2020: 34,608; 2021: 43,075; 2022: 43,653; 2023: 40,109;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="51" t="inlineStr">
+        <is>
+          <t>2024: 41,950; 2025: 44,328. Adjusted EPS 2019: 3.24; 2020: 3.65; 2021: 5.21; 2022: 5.34; 2023: 4.44; 2024: 4.67; 2025: 5.15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="51" t="inlineStr">
+        <is>
+          <t>FY2025 quarterly adj. EPS: 1.09 / 1.26 / 1.30 / 1.50. Q1'26: net sales 11,164; adj. EPS 1.15; comparable growth +3.7%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="51" t="inlineStr">
+        <is>
+          <t>Caveats: the FY2026 sales 'required remaining growth' weights quarters by prior-year REPORTED sales (Abbott's comparable</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="51" t="inlineStr">
+        <is>
+          <t>base also nets out the Exact Sciences acquisition and FX, which I don't have at quarterly granularity) - treat as indicative;</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="51" t="inlineStr">
+        <is>
+          <t>the EPS calculator is exact. FY2020 total-company organic % and FY2022/FY2023 some organic splits were not cleanly</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="51" t="inlineStr">
+        <is>
+          <t>confirmed and are left blank rather than estimated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="52" t="inlineStr">
+        <is>
+          <t>PRIMARY SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="51" t="inlineStr">
+        <is>
+          <t>Abbott investor news (abbott.mediaroom.com) and PR Newswire press releases, plus the corresponding SEC 8-K exhibit 99.1 for</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="51" t="inlineStr">
+        <is>
+          <t>each quarter. Per-row source links are in the 'Source' column of the Guidance Timeline sheet. Secondary cross-checks included</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="51" t="inlineStr">
+        <is>
+          <t>Nasdaq, StockTitan, RTTNews, MedTech Dive, 360Dx, Motley Fool / Seeking Alpha transcripts and Investing.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="51" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="51" t="inlineStr">
+        <is>
+          <t>Compiled 2026-06-05. Figures are guidance as issued at the time of each report, not actuals. For an auditable record, confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="51" t="inlineStr">
+        <is>
+          <t>each figure against the linked SEC 8-K / press release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="53" t="inlineStr">
+        <is>
+          <t>ACTION COLOR LEGEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="54" t="n"/>
+      <c r="B62" s="55" t="inlineStr">
+        <is>
+          <t>Initial — Initial outlook for a fiscal year</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="56" t="n"/>
+      <c r="B63" s="55" t="inlineStr">
+        <is>
+          <t>Raised — Guidance raised vs prior update</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="57" t="n"/>
+      <c r="B64" s="55" t="inlineStr">
+        <is>
+          <t>Maintained — Held or reaffirmed around the same level</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="57" t="n"/>
+      <c r="B65" s="55" t="inlineStr">
+        <is>
+          <t>Narrowed (midpoint raised) — Range tightened, midpoint up</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="58" t="n"/>
+      <c r="B66" s="55" t="inlineStr">
+        <is>
+          <t>Reinstated (floor) — Guidance restored as an 'at least' floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="59" t="n"/>
+      <c r="B67" s="55" t="inlineStr">
+        <is>
+          <t>Lowered — Guidance reduced vs prior update</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="60" t="n"/>
+      <c r="B68" s="55" t="inlineStr">
+        <is>
+          <t>Withdrawn — Guidance suspended</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="53" t="inlineStr">
+        <is>
+          <t>SALES GROWTH BASIS COLOR LEGEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="56" t="n"/>
+      <c r="B71" s="55" t="inlineStr">
+        <is>
+          <t>Total-company organic — Clean organic % for the whole company</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="56" t="n"/>
+      <c r="B72" s="55" t="inlineStr">
+        <is>
+          <t>Organic (COVID immaterial) — Single organic range, COVID negligible (FY2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="61" t="n"/>
+      <c r="B73" s="55" t="inlineStr">
+        <is>
+          <t>Organic, ex-COVID — Organic excluding residual COVID testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="57" t="n"/>
+      <c r="B74" s="55" t="inlineStr">
+        <is>
+          <t>Base business, ex-COVID testing — Underlying growth ex-COVID (often a descriptor, 2021-2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="54" t="n"/>
+      <c r="B75" s="55" t="inlineStr">
+        <is>
+          <t>Comparable (adj. for M&amp;A &amp; FX) — Adjusted for the Exact Sciences acquisition &amp; FX (FY2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="60" t="n"/>
+      <c r="B76" s="55" t="inlineStr">
+        <is>
+          <t>Not quantified — No sales-growth figure issued</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>